<commit_message>
PSP-10909 fixes on document types following sentence case format
</commit_message>
<xml_diff>
--- a/tools/mayan_sync_helper/xml_definitions/doctype_definitions.xlsx
+++ b/tools/mayan_sync_helper/xml_definitions/doctype_definitions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SueT\projects\PSP\tools\mayan_sync_helper\xml_definitions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1EC5009-899C-4B6C-B378-FE7BDC77102A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D513DC9-39D7-4033-9578-0A6A399016FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{B36D4D41-52C3-4254-819B-044EB561F7B6}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{B36D4D41-52C3-4254-819B-044EB561F7B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="215">
   <si>
     <t>Document type</t>
   </si>
@@ -370,18 +370,6 @@
     <t>Research File</t>
   </si>
   <si>
-    <t>Purchase and Sale Agreement</t>
-  </si>
-  <si>
-    <t>Enhanced Referral Records</t>
-  </si>
-  <si>
-    <t>Certificate of Compliance</t>
-  </si>
-  <si>
-    <t>First Nations Strength of Claim Report</t>
-  </si>
-  <si>
     <t>FNSCR</t>
   </si>
   <si>
@@ -400,9 +388,6 @@
     <t>ALC</t>
   </si>
   <si>
-    <t>Agricultural Land Commission (ALC)</t>
-  </si>
-  <si>
     <t>FORM12</t>
   </si>
   <si>
@@ -412,15 +397,9 @@
     <t>LANDACTTENRES</t>
   </si>
   <si>
-    <t>Land Act Tenure/Reserves</t>
-  </si>
-  <si>
     <t>Purpose</t>
   </si>
   <si>
-    <t>Form 5 - Approval of expropriation</t>
-  </si>
-  <si>
     <t>The Approval of Expropriation (Form 5) for Expropriations</t>
   </si>
   <si>
@@ -622,139 +601,88 @@
     <t>WAIVECONDS</t>
   </si>
   <si>
-    <t>Briefing/Decision notes</t>
-  </si>
-  <si>
-    <t>Affidavit of Service</t>
-  </si>
-  <si>
-    <t>BC Assessment Search</t>
-  </si>
-  <si>
-    <t>Canada Lands Survey</t>
-  </si>
-  <si>
     <t>CDOGS Template</t>
   </si>
   <si>
-    <t>Compensation Cheque</t>
-  </si>
-  <si>
-    <t>Compensation Requisition (H-120)</t>
-  </si>
-  <si>
-    <t>Company Search</t>
-  </si>
-  <si>
-    <t>Condition of Entry (H0443)</t>
-  </si>
-  <si>
-    <t>Conveyance Closing Documents (ex: PTT forms, Form A transfer etc.)</t>
-  </si>
-  <si>
-    <t>Crown Grant</t>
-  </si>
-  <si>
-    <t>District Road Register</t>
-  </si>
-  <si>
-    <t>Field Notes</t>
-  </si>
-  <si>
-    <t>Financial Records (invoices, journal vouchers, received cheques etc.)</t>
-  </si>
-  <si>
-    <t>First Nations Consultation</t>
-  </si>
-  <si>
-    <t>Historical File</t>
-  </si>
-  <si>
-    <t>Lease / License Agreement</t>
-  </si>
-  <si>
-    <t>Legal Correspondence (ex: to AG/external lawyers)</t>
-  </si>
-  <si>
-    <t>Legal Survey Plan</t>
-  </si>
-  <si>
-    <t>Letter of Intent</t>
-  </si>
-  <si>
-    <t>Approval/Sign-off</t>
-  </si>
-  <si>
-    <t>Listing Agreement</t>
-  </si>
-  <si>
-    <t>LTSA Documents and Plans (except title search)</t>
-  </si>
-  <si>
-    <t>Ministerial Order</t>
-  </si>
-  <si>
-    <t>Miscellaneous Notes (LTSA)</t>
-  </si>
-  <si>
-    <t>MoTT Plan</t>
-  </si>
-  <si>
-    <t>Form 7 - Notice of Abandonement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Form 8 - Notice of Advanced Payment </t>
-  </si>
-  <si>
-    <t>Notice of Claims/Litigation Documents</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Form 1 - Notice of Expropriation </t>
-  </si>
-  <si>
-    <t>Notice of Possible Entry (H0224)</t>
-  </si>
-  <si>
-    <t>Owner Agreement/Offer</t>
-  </si>
-  <si>
-    <t>PA Plans / Design Drawings</t>
-  </si>
-  <si>
-    <t>Privy Council</t>
-  </si>
-  <si>
-    <t>Professional Reports (ex: engineering/environmental etc.)</t>
-  </si>
-  <si>
-    <t>Record of Negotiation</t>
-  </si>
-  <si>
-    <t>Release of Claims</t>
-  </si>
-  <si>
-    <t>Surplus Property Declaration</t>
-  </si>
-  <si>
-    <t>Tax Notices and Assessments</t>
-  </si>
-  <si>
-    <t>Temporary License for Construction Access (H0074)</t>
-  </si>
-  <si>
-    <t>Term Sheet/Offer</t>
-  </si>
-  <si>
-    <t>Title Search / Historical Title</t>
-  </si>
-  <si>
-    <t>Transfer of Administration</t>
-  </si>
-  <si>
-    <t>Form 9 - Vesting Notice (Form 9)</t>
-  </si>
-  <si>
-    <t>Waiver of Conditions</t>
+    <t>Agricultural land commission (ALC)</t>
+  </si>
+  <si>
+    <t>Form 5 - approval of expropriation</t>
+  </si>
+  <si>
+    <t>Briefing/ Decision notes</t>
+  </si>
+  <si>
+    <t>Certificate of compliance</t>
+  </si>
+  <si>
+    <t>Certificate of insurance (H0111)</t>
+  </si>
+  <si>
+    <t>Order in council (OIC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Form 1 - Notice of expropriation </t>
+  </si>
+  <si>
+    <t>Notice of claims/ Litigation documents</t>
+  </si>
+  <si>
+    <t>Enhanced referral records</t>
+  </si>
+  <si>
+    <t>Financial records (invoices, journal vouchers, received cheques etc.)</t>
+  </si>
+  <si>
+    <t>First nations strength of claim report</t>
+  </si>
+  <si>
+    <t>Land act tenure/ Reserves</t>
+  </si>
+  <si>
+    <t>Lease / License agreement</t>
+  </si>
+  <si>
+    <t>Approval/ Sign-off</t>
+  </si>
+  <si>
+    <t>Listing agreement</t>
+  </si>
+  <si>
+    <t>MoTT plan</t>
+  </si>
+  <si>
+    <t>Form 7 - Notice of abandonement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Form 8 - Notice of advanced payment </t>
+  </si>
+  <si>
+    <t>Other Land Agreement (Indemnity Letter, Letter of intended use, Assumption agreement, etc)</t>
+  </si>
+  <si>
+    <t>Owner agreement/ Offer</t>
+  </si>
+  <si>
+    <t>Purchase and sale agreement</t>
+  </si>
+  <si>
+    <t>Spending authority approval (SAA)</t>
+  </si>
+  <si>
+    <t>Term sheet/ Offer</t>
+  </si>
+  <si>
+    <t>Title search/ Historical title</t>
+  </si>
+  <si>
+    <t>Utility bills</t>
+  </si>
+  <si>
+    <t>Form 9 - Vesting notice (Form 9)</t>
+  </si>
+  <si>
+    <t>Waiver of conditions</t>
   </si>
 </sst>
 </file>
@@ -1595,21 +1523,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{136C655F-10D5-4146-8405-A6BFCE94F80F}">
   <dimension ref="B2:J65"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="57.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" customWidth="1"/>
-    <col min="7" max="7" width="19.85546875" customWidth="1"/>
-    <col min="8" max="8" width="18.5703125" customWidth="1"/>
-    <col min="9" max="9" width="20.140625" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="57.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" customWidth="1"/>
+    <col min="6" max="6" width="17.6640625" customWidth="1"/>
+    <col min="7" max="7" width="19.88671875" customWidth="1"/>
+    <col min="8" max="8" width="18.5546875" customWidth="1"/>
+    <col min="9" max="9" width="20.109375" customWidth="1"/>
     <col min="10" max="10" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>107</v>
       </c>
@@ -1617,7 +1545,7 @@
         <v>108</v>
       </c>
       <c r="D2" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="E2" t="s">
         <v>1</v>
@@ -1635,18 +1563,18 @@
         <v>5</v>
       </c>
       <c r="J2" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="3" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B3" s="4" t="s">
         <v>91</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>195</v>
+        <v>41</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
@@ -1659,15 +1587,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>120</v>
+        <v>188</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
@@ -1680,15 +1608,15 @@
       </c>
       <c r="J4" s="7"/>
     </row>
-    <row r="5" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>89</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>126</v>
+        <v>189</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
@@ -1701,7 +1629,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B6" s="4" t="s">
         <v>79</v>
       </c>
@@ -1709,7 +1637,7 @@
         <v>29</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
@@ -1726,15 +1654,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B7" s="4" t="s">
         <v>73</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>196</v>
+        <v>6</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="7" t="s">
@@ -1753,15 +1681,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
         <v>98</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>7</v>
@@ -1782,15 +1710,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B9" s="4" t="s">
         <v>70</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>197</v>
+        <v>23</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="7" t="s">
@@ -1807,15 +1735,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
         <v>104</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
@@ -1826,15 +1754,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B11" s="4" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>112</v>
+        <v>191</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
@@ -1847,15 +1775,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B12" s="4" t="s">
         <v>96</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>46</v>
+        <v>192</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
@@ -1870,15 +1798,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B13" s="4" t="s">
         <v>84</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>199</v>
+        <v>34</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="E13" s="7"/>
       <c r="F13" s="7"/>
@@ -1891,15 +1819,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B14" s="4" t="s">
         <v>83</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>200</v>
+        <v>33</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
@@ -1914,15 +1842,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B15" s="4" t="s">
         <v>77</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>201</v>
+        <v>27</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="E15" s="7"/>
       <c r="F15" s="7" t="s">
@@ -1941,15 +1869,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B16" s="4" t="s">
         <v>85</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="E16" s="7"/>
       <c r="F16" s="7" t="s">
@@ -1964,15 +1892,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="2:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B17" s="4" t="s">
         <v>101</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>203</v>
+        <v>51</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
@@ -1989,7 +1917,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B18" s="4" t="s">
         <v>65</v>
       </c>
@@ -1997,7 +1925,7 @@
         <v>22</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>7</v>
@@ -2018,15 +1946,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B19" s="4" t="s">
         <v>63</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>204</v>
+        <v>21</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="E19" s="7"/>
       <c r="F19" s="7" t="s">
@@ -2041,15 +1969,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B20" s="4" t="s">
         <v>74</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>205</v>
+        <v>20</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="E20" s="7"/>
       <c r="F20" s="7" t="s">
@@ -2064,15 +1992,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B21" s="4" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>111</v>
+        <v>196</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="E21" s="7"/>
       <c r="F21" s="7"/>
@@ -2085,15 +2013,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B22" s="4" t="s">
         <v>75</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>206</v>
+        <v>19</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="7" t="s">
@@ -2110,15 +2038,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="2:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B23" s="4" t="s">
         <v>105</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>7</v>
@@ -2139,15 +2067,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B24" s="4" t="s">
         <v>93</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>208</v>
+        <v>43</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="E24" s="7"/>
       <c r="F24" s="7" t="s">
@@ -2166,15 +2094,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B25" s="4" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>113</v>
+        <v>198</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="E25" s="7"/>
       <c r="F25" s="7"/>
@@ -2189,15 +2117,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B26" s="4" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="E26" s="7"/>
       <c r="F26" s="7" t="s">
@@ -2216,7 +2144,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B27" s="4" t="s">
         <v>58</v>
       </c>
@@ -2224,7 +2152,7 @@
         <v>18</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="E27" s="7"/>
       <c r="F27" s="7" t="s">
@@ -2243,15 +2171,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B28" s="4" t="s">
         <v>64</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>209</v>
+        <v>17</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="E28" s="7" t="s">
         <v>7</v>
@@ -2272,15 +2200,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B29" s="4" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>124</v>
+        <v>199</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="E29" s="7"/>
       <c r="F29" s="7"/>
@@ -2291,15 +2219,15 @@
       <c r="I29" s="7"/>
       <c r="J29" s="7"/>
     </row>
-    <row r="30" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B30" s="4" t="s">
         <v>57</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="E30" s="7"/>
       <c r="F30" s="7" t="s">
@@ -2316,15 +2244,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B31" s="4" t="s">
         <v>102</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>211</v>
+        <v>52</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="E31" s="7" t="s">
         <v>7</v>
@@ -2345,15 +2273,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B32" s="4" t="s">
         <v>60</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>212</v>
+        <v>16</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="E32" s="7" t="s">
         <v>7</v>
@@ -2374,15 +2302,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B33" s="4" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>213</v>
+        <v>183</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="E33" s="7"/>
       <c r="F33" s="7"/>
@@ -2393,15 +2321,15 @@
       </c>
       <c r="J33" s="7"/>
     </row>
-    <row r="34" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B34" s="4" t="s">
         <v>97</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>214</v>
+        <v>201</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="E34" s="7"/>
       <c r="F34" s="7"/>
@@ -2414,15 +2342,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B35" s="4" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>215</v>
+        <v>202</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="E35" s="7"/>
       <c r="F35" s="7"/>
@@ -2433,15 +2361,15 @@
       </c>
       <c r="J35" s="7"/>
     </row>
-    <row r="36" spans="2:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B36" s="4" t="s">
         <v>78</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>216</v>
+        <v>28</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="E36" s="7"/>
       <c r="F36" s="7" t="s">
@@ -2460,15 +2388,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B37" s="4" t="s">
         <v>71</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>217</v>
+        <v>15</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="E37" s="7"/>
       <c r="F37" s="7" t="s">
@@ -2483,15 +2411,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B38" s="4" t="s">
         <v>67</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>218</v>
+        <v>14</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="E38" s="7"/>
       <c r="F38" s="7" t="s">
@@ -2510,15 +2438,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B39" s="4" t="s">
         <v>59</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>219</v>
+        <v>203</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="E39" s="7" t="s">
         <v>7</v>
@@ -2539,12 +2467,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B40" s="4" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>220</v>
+        <v>204</v>
       </c>
       <c r="D40" s="6"/>
       <c r="E40" s="7"/>
@@ -2556,15 +2484,15 @@
       <c r="I40" s="7"/>
       <c r="J40" s="7"/>
     </row>
-    <row r="41" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B41" s="4" t="s">
         <v>86</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="E41" s="7"/>
       <c r="F41" s="7"/>
@@ -2577,15 +2505,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B42" s="4" t="s">
         <v>95</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>222</v>
+        <v>195</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="E42" s="7"/>
       <c r="F42" s="7" t="s">
@@ -2600,15 +2528,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B43" s="4" t="s">
         <v>88</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>223</v>
+        <v>194</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="E43" s="7"/>
       <c r="F43" s="7"/>
@@ -2621,15 +2549,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B44" s="4" t="s">
         <v>92</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>224</v>
+        <v>42</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="E44" s="7"/>
       <c r="F44" s="7" t="s">
@@ -2644,15 +2572,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B45" s="4" t="s">
         <v>61</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>12</v>
+        <v>193</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="E45" s="7"/>
       <c r="F45" s="7" t="s">
@@ -2669,7 +2597,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B46" s="4" t="s">
         <v>76</v>
       </c>
@@ -2677,7 +2605,7 @@
         <v>11</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="E46" s="7" t="s">
         <v>7</v>
@@ -2698,15 +2626,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="47" spans="2:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B47" s="4" t="s">
         <v>106</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>54</v>
+        <v>206</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
@@ -2723,15 +2651,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="2:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B48" s="4" t="s">
         <v>82</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>225</v>
+        <v>207</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="E48" s="7"/>
       <c r="F48" s="7" t="s">
@@ -2746,15 +2674,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B49" s="4" t="s">
         <v>56</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>226</v>
+        <v>10</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="E49" s="7" t="s">
         <v>7</v>
@@ -2771,7 +2699,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B50" s="4" t="s">
         <v>68</v>
       </c>
@@ -2779,7 +2707,7 @@
         <v>69</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="E50" s="7" t="s">
         <v>7</v>
@@ -2800,15 +2728,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B51" s="4" t="s">
         <v>62</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>227</v>
+        <v>8</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="E51" s="7"/>
       <c r="F51" s="7" t="s">
@@ -2823,15 +2751,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="2:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B52" s="4" t="s">
         <v>80</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>228</v>
+        <v>30</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="E52" s="7"/>
       <c r="F52" s="7" t="s">
@@ -2850,15 +2778,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="53" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B53" s="4" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>110</v>
+        <v>208</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="E53" s="7"/>
       <c r="F53" s="7"/>
@@ -2871,15 +2799,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B54" s="4" t="s">
         <v>103</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>229</v>
+        <v>53</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="E54" s="7"/>
       <c r="F54" s="7"/>
@@ -2894,15 +2822,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B55" s="4" t="s">
         <v>87</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>230</v>
+        <v>37</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="E55" s="7"/>
       <c r="F55" s="7"/>
@@ -2917,15 +2845,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="56" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B56" s="4" t="s">
         <v>81</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>31</v>
+        <v>209</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="E56" s="7" t="s">
         <v>7</v>
@@ -2942,15 +2870,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="57" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B57" s="4" t="s">
         <v>99</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>231</v>
+        <v>49</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="E57" s="7" t="s">
         <v>7</v>
@@ -2969,15 +2897,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="58" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B58" s="4" t="s">
         <v>94</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>232</v>
+        <v>44</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="E58" s="7"/>
       <c r="F58" s="7" t="s">
@@ -2996,15 +2924,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="59" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B59" s="4" t="s">
         <v>100</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>233</v>
+        <v>50</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="E59" s="7"/>
       <c r="F59" s="7"/>
@@ -3017,15 +2945,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="60" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B60" s="4" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>234</v>
+        <v>210</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="E60" s="7"/>
       <c r="F60" s="7"/>
@@ -3036,15 +2964,15 @@
       <c r="I60" s="7"/>
       <c r="J60" s="7"/>
     </row>
-    <row r="61" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B61" s="4" t="s">
         <v>66</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>235</v>
+        <v>211</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="E61" s="7"/>
       <c r="F61" s="7" t="s">
@@ -3063,15 +2991,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B62" s="4" t="s">
         <v>72</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>236</v>
+        <v>25</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="E62" s="7"/>
       <c r="F62" s="7" t="s">
@@ -3090,15 +3018,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B63" s="4" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>186</v>
+        <v>212</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="E63" s="7"/>
       <c r="F63" s="7"/>
@@ -3109,15 +3037,15 @@
       <c r="I63" s="7"/>
       <c r="J63" s="7"/>
     </row>
-    <row r="64" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B64" s="8" t="s">
         <v>90</v>
       </c>
       <c r="C64" s="9" t="s">
-        <v>237</v>
+        <v>213</v>
       </c>
       <c r="D64" s="10" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="E64" s="11"/>
       <c r="F64" s="11"/>
@@ -3130,12 +3058,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:10" x14ac:dyDescent="0.3">
       <c r="B65" s="8" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="C65" s="9" t="s">
-        <v>238</v>
+        <v>214</v>
       </c>
       <c r="D65" s="10"/>
       <c r="E65" s="11"/>
@@ -3163,15 +3091,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB6CFB30-CB71-47BC-BF9F-44CEDC4A3FFF}">
   <dimension ref="B1:G52"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="42.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="2" max="2" width="42.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
@@ -3179,7 +3107,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="2:7" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:7" ht="51" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
@@ -3199,7 +3127,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>41</v>
       </c>
@@ -3213,7 +3141,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
         <v>29</v>
       </c>
@@ -3229,7 +3157,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>39</v>
       </c>
@@ -3241,7 +3169,7 @@
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
     </row>
-    <row r="7" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>6</v>
       </c>
@@ -3259,7 +3187,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>48</v>
       </c>
@@ -3279,7 +3207,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>23</v>
       </c>
@@ -3297,7 +3225,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
         <v>46</v>
       </c>
@@ -3313,7 +3241,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
         <v>27</v>
       </c>
@@ -3331,7 +3259,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>34</v>
       </c>
@@ -3345,7 +3273,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
         <v>33</v>
       </c>
@@ -3359,7 +3287,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="3" t="s">
         <v>35</v>
       </c>
@@ -3373,7 +3301,7 @@
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
     </row>
-    <row r="15" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
         <v>51</v>
       </c>
@@ -3387,7 +3315,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="3" t="s">
         <v>22</v>
       </c>
@@ -3407,7 +3335,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="3" t="s">
         <v>21</v>
       </c>
@@ -3423,7 +3351,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="3" t="s">
         <v>20</v>
       </c>
@@ -3439,7 +3367,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19" s="3" t="s">
         <v>19</v>
       </c>
@@ -3455,7 +3383,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="3" t="s">
         <v>55</v>
       </c>
@@ -3475,7 +3403,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="3" t="s">
         <v>43</v>
       </c>
@@ -3493,7 +3421,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
         <v>18</v>
       </c>
@@ -3511,7 +3439,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="3" t="s">
         <v>17</v>
       </c>
@@ -3531,7 +3459,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="3" t="s">
         <v>26</v>
       </c>
@@ -3549,7 +3477,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="3" t="s">
         <v>52</v>
       </c>
@@ -3569,7 +3497,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="3" t="s">
         <v>16</v>
       </c>
@@ -3589,7 +3517,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="3" t="s">
         <v>47</v>
       </c>
@@ -3601,7 +3529,7 @@
       </c>
       <c r="G27" s="3"/>
     </row>
-    <row r="28" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="3" t="s">
         <v>28</v>
       </c>
@@ -3619,7 +3547,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
         <v>15</v>
       </c>
@@ -3635,7 +3563,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B30" s="3" t="s">
         <v>14</v>
       </c>
@@ -3653,7 +3581,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="3" t="s">
         <v>13</v>
       </c>
@@ -3673,7 +3601,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="3" t="s">
         <v>36</v>
       </c>
@@ -3685,7 +3613,7 @@
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
     </row>
-    <row r="33" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B33" s="3" t="s">
         <v>45</v>
       </c>
@@ -3701,7 +3629,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B34" s="3" t="s">
         <v>38</v>
       </c>
@@ -3713,7 +3641,7 @@
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
     </row>
-    <row r="35" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="3" t="s">
         <v>42</v>
       </c>
@@ -3727,7 +3655,7 @@
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
     </row>
-    <row r="36" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B36" s="3" t="s">
         <v>12</v>
       </c>
@@ -3743,7 +3671,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="37" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="3" t="s">
         <v>11</v>
       </c>
@@ -3763,7 +3691,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:7" ht="51" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B38" s="3" t="s">
         <v>54</v>
       </c>
@@ -3779,7 +3707,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B39" s="3" t="s">
         <v>32</v>
       </c>
@@ -3795,7 +3723,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B40" s="3" t="s">
         <v>10</v>
       </c>
@@ -3813,7 +3741,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="3" t="s">
         <v>9</v>
       </c>
@@ -3833,7 +3761,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="3" t="s">
         <v>8</v>
       </c>
@@ -3847,7 +3775,7 @@
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
     </row>
-    <row r="43" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B43" s="3" t="s">
         <v>30</v>
       </c>
@@ -3865,7 +3793,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B44" s="3" t="s">
         <v>53</v>
       </c>
@@ -3879,7 +3807,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B45" s="3" t="s">
         <v>37</v>
       </c>
@@ -3891,7 +3819,7 @@
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
     </row>
-    <row r="46" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B46" s="3" t="s">
         <v>31</v>
       </c>
@@ -3909,7 +3837,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="47" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B47" s="3" t="s">
         <v>49</v>
       </c>
@@ -3927,7 +3855,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B48" s="3" t="s">
         <v>44</v>
       </c>
@@ -3945,7 +3873,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B49" s="3" t="s">
         <v>50</v>
       </c>
@@ -3957,7 +3885,7 @@
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
     </row>
-    <row r="50" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B50" s="3" t="s">
         <v>24</v>
       </c>
@@ -3975,7 +3903,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B51" s="3" t="s">
         <v>25</v>
       </c>
@@ -3991,7 +3919,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B52" s="3" t="s">
         <v>40</v>
       </c>
@@ -4012,13 +3940,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1355EE7-9C2F-4813-B2F0-184BA37951AC}">
   <dimension ref="B1:G51"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="32.85546875" customWidth="1"/>
+    <col min="2" max="2" width="32.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="3"/>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4026,7 +3954,7 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3" t="s">
         <v>41</v>
       </c>
@@ -4040,7 +3968,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>29</v>
       </c>
@@ -4056,7 +3984,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
         <v>39</v>
       </c>
@@ -4068,7 +3996,7 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
     </row>
-    <row r="6" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
@@ -4086,7 +4014,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>48</v>
       </c>
@@ -4106,7 +4034,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B8" s="3" t="s">
         <v>23</v>
       </c>
@@ -4124,7 +4052,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>46</v>
       </c>
@@ -4140,7 +4068,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
         <v>27</v>
       </c>
@@ -4158,7 +4086,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
         <v>34</v>
       </c>
@@ -4172,7 +4100,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B12" s="3" t="s">
         <v>33</v>
       </c>
@@ -4186,7 +4114,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
         <v>35</v>
       </c>
@@ -4200,7 +4128,7 @@
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
     </row>
-    <row r="14" spans="2:7" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:7" ht="51" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="3" t="s">
         <v>51</v>
       </c>
@@ -4214,7 +4142,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="3" t="s">
         <v>22</v>
       </c>
@@ -4234,7 +4162,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="3" t="s">
         <v>21</v>
       </c>
@@ -4250,7 +4178,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B17" s="3" t="s">
         <v>20</v>
       </c>
@@ -4266,7 +4194,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="3" t="s">
         <v>19</v>
       </c>
@@ -4282,7 +4210,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19" s="3" t="s">
         <v>55</v>
       </c>
@@ -4302,7 +4230,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B20" s="3" t="s">
         <v>43</v>
       </c>
@@ -4320,7 +4248,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B21" s="3" t="s">
         <v>18</v>
       </c>
@@ -4338,7 +4266,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B22" s="3" t="s">
         <v>17</v>
       </c>
@@ -4358,7 +4286,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B23" s="3" t="s">
         <v>26</v>
       </c>
@@ -4376,7 +4304,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B24" s="3" t="s">
         <v>52</v>
       </c>
@@ -4396,7 +4324,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B25" s="3" t="s">
         <v>16</v>
       </c>
@@ -4416,7 +4344,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B26" s="3" t="s">
         <v>47</v>
       </c>
@@ -4428,7 +4356,7 @@
       </c>
       <c r="G26" s="3"/>
     </row>
-    <row r="27" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="3" t="s">
         <v>28</v>
       </c>
@@ -4446,7 +4374,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B28" s="3" t="s">
         <v>15</v>
       </c>
@@ -4462,7 +4390,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B29" s="3" t="s">
         <v>14</v>
       </c>
@@ -4480,7 +4408,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B30" s="3" t="s">
         <v>13</v>
       </c>
@@ -4500,7 +4428,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B31" s="3" t="s">
         <v>36</v>
       </c>
@@ -4512,7 +4440,7 @@
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
     </row>
-    <row r="32" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B32" s="3" t="s">
         <v>45</v>
       </c>
@@ -4528,7 +4456,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B33" s="3" t="s">
         <v>38</v>
       </c>
@@ -4540,7 +4468,7 @@
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
     </row>
-    <row r="34" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B34" s="3" t="s">
         <v>42</v>
       </c>
@@ -4554,7 +4482,7 @@
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
     </row>
-    <row r="35" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="3" t="s">
         <v>12</v>
       </c>
@@ -4570,7 +4498,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B36" s="3" t="s">
         <v>11</v>
       </c>
@@ -4590,7 +4518,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="37" spans="2:7" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:7" ht="67.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B37" s="3" t="s">
         <v>54</v>
       </c>
@@ -4606,7 +4534,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B38" s="3" t="s">
         <v>32</v>
       </c>
@@ -4622,7 +4550,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B39" s="3" t="s">
         <v>10</v>
       </c>
@@ -4640,7 +4568,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B40" s="3" t="s">
         <v>9</v>
       </c>
@@ -4660,7 +4588,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B41" s="3" t="s">
         <v>8</v>
       </c>
@@ -4674,7 +4602,7 @@
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
     </row>
-    <row r="42" spans="2:7" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B42" s="3" t="s">
         <v>30</v>
       </c>
@@ -4692,7 +4620,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B43" s="3" t="s">
         <v>53</v>
       </c>
@@ -4706,7 +4634,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B44" s="3" t="s">
         <v>37</v>
       </c>
@@ -4718,7 +4646,7 @@
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
     </row>
-    <row r="45" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B45" s="3" t="s">
         <v>31</v>
       </c>
@@ -4736,7 +4664,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B46" s="3" t="s">
         <v>49</v>
       </c>
@@ -4754,7 +4682,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="47" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B47" s="3" t="s">
         <v>44</v>
       </c>
@@ -4772,7 +4700,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="2:7" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:7" ht="34.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B48" s="3" t="s">
         <v>50</v>
       </c>
@@ -4784,7 +4712,7 @@
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
     </row>
-    <row r="49" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B49" s="3" t="s">
         <v>24</v>
       </c>
@@ -4802,7 +4730,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="50" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B50" s="3" t="s">
         <v>25</v>
       </c>
@@ -4818,7 +4746,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B51" s="3" t="s">
         <v>40</v>
       </c>

</xml_diff>